<commit_message>
updates after rev notes
</commit_message>
<xml_diff>
--- a/model_accu_scores.xlsx
+++ b/model_accu_scores.xlsx
@@ -478,25 +478,25 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.837</v>
+        <v>0.95</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.986</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.923</v>
+        <v>0.957</v>
       </c>
       <c r="H2" t="n">
-        <v>0.994</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0.994</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -504,28 +504,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.837</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
         <v>0.993</v>
       </c>
-      <c r="F3" t="n">
-        <v>0.973</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.964</v>
-      </c>
       <c r="H3" t="n">
-        <v>0.966</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0.987</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -533,28 +533,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0.991</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.757</v>
+        <v>0.843</v>
       </c>
       <c r="D4" t="n">
-        <v>0.996</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>0.803</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.996</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0.844</v>
+        <v>0.921</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0.984</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -562,28 +562,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>0.974</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.737</v>
+        <v>0.886</v>
       </c>
       <c r="D5" t="n">
-        <v>0.996</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>0.82</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.971</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.866</v>
+        <v>0.929</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>0.986</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>